<commit_message>
ABP Demo-Test Suite execution
</commit_message>
<xml_diff>
--- a/KatalonData/ABPTestData/SchedulePaymentABP_NoCF.xlsx
+++ b/KatalonData/ABPTestData/SchedulePaymentABP_NoCF.xlsx
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="57">
   <si>
     <t>Result</t>
   </si>
@@ -287,6 +287,18 @@
   </si>
   <si>
     <t>Fri Jun 19 12:52:18 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jul 24 22:46:30 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jul 24 22:48:34 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jul 24 22:51:25 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jul 24 22:54:16 IST 2026</t>
   </si>
 </sst>
 </file>
@@ -669,7 +681,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="11" max="11" customWidth="true" width="23.54296875" collapsed="true"/>
@@ -697,13 +709,13 @@
       <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" t="s" s="0">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" t="s" s="0">
         <v>9</v>
       </c>
       <c r="K1" s="3" t="s">
@@ -726,10 +738,10 @@
       </c>
     </row>
     <row ht="409.5" r="2" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>14</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>52</v>
       </c>
       <c r="C2" s="4"/>
@@ -742,17 +754,17 @@
       <c r="F2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="G2" t="str">
+      <c r="G2" t="str" s="0">
         <f>"CarlosJacinta"</f>
         <v>CarlosJacinta</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" t="s" s="0">
         <v>18</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" t="s" s="0">
         <v>20</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" t="s" s="0">
         <v>19</v>
       </c>
       <c r="K2" s="6" t="s">
@@ -815,7 +827,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49CD28ED-6B88-4076-A023-4B2AA175CC49}">
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" bestFit="true" customWidth="true" width="5.6328125" collapsed="true"/>
@@ -845,13 +857,13 @@
       <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" t="s" s="0">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" t="s" s="0">
         <v>9</v>
       </c>
       <c r="K1" s="3" t="s">
@@ -874,10 +886,10 @@
       </c>
     </row>
     <row ht="409.5" r="2" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>14</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>49</v>
       </c>
       <c r="C2" s="4"/>
@@ -890,17 +902,17 @@
       <c r="F2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="G2" t="str">
+      <c r="G2" t="str" s="0">
         <f>"Bridges"</f>
         <v>Bridges</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" t="s" s="0">
         <v>18</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" t="s" s="0">
         <v>20</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" t="s" s="0">
         <v>19</v>
       </c>
       <c r="K2" s="6" t="s">
@@ -959,7 +971,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A38E6C38-F14D-4B06-9F0D-017FEF3E0BF1}">
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="11" max="11" customWidth="true" width="32.90625" collapsed="true"/>
@@ -987,13 +999,13 @@
       <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" t="s" s="0">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" t="s" s="0">
         <v>9</v>
       </c>
       <c r="K1" s="3" t="s">
@@ -1016,11 +1028,11 @@
       </c>
     </row>
     <row ht="409.5" r="2" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>14</v>
       </c>
-      <c r="B2" t="s">
-        <v>51</v>
+      <c r="B2" t="s" s="0">
+        <v>56</v>
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="5" t="s">
@@ -1032,17 +1044,17 @@
       <c r="F2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="G2" t="str">
+      <c r="G2" t="str" s="0">
         <f>"Carlos"</f>
         <v>Carlos</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" t="s" s="0">
         <v>18</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" t="s" s="0">
         <v>20</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" t="s" s="0">
         <v>19</v>
       </c>
       <c r="K2" s="6" t="s">
@@ -1102,7 +1114,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BACB12DE-9459-4B21-A76D-74D1C2CFA77A}">
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="11" max="11" customWidth="true" width="20.81640625" collapsed="true"/>
@@ -1130,13 +1142,13 @@
       <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" t="s" s="0">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" t="s" s="0">
         <v>9</v>
       </c>
       <c r="K1" s="3" t="s">
@@ -1159,11 +1171,11 @@
       </c>
     </row>
     <row ht="409.5" r="2" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>14</v>
       </c>
-      <c r="B2" t="s">
-        <v>50</v>
+      <c r="B2" t="s" s="0">
+        <v>54</v>
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="5" t="s">
@@ -1175,17 +1187,17 @@
       <c r="F2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="G2" t="str">
+      <c r="G2" t="str" s="0">
         <f>"Smith"</f>
         <v>Smith</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" t="s" s="0">
         <v>18</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" t="s" s="0">
         <v>20</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" t="s" s="0">
         <v>19</v>
       </c>
       <c r="K2" s="6" t="s">

</xml_diff>